<commit_message>
feat(Claude): Aset Hak Guna — masa sewa bulan, frekuensi bayar, tahun buku, fiskal akrual + laporan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UpjcfzeoGGmyCzxVY4c69u
</commit_message>
<xml_diff>
--- a/tools/aset-hak-guna/Template-Isian-Aset-Hak-Guna.xlsx
+++ b/tools/aset-hak-guna/Template-Isian-Aset-Hak-Guna.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petunjuk" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Input'!$A$1:$C$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Input'!$A$1:$C$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -672,187 +672,207 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Masa sewa (tahun)</t>
+          <t>Masa sewa (bulan)</t>
         </is>
       </c>
       <c r="B15" s="11" t="n"/>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Lama sewa sesuai kontrak, termasuk perpanjangan yang hampir pasti diambil</t>
+          <t>Lama sewa dalam BULAN sesuai kontrak, termasuk perpanjangan yang hampir pasti diambil. Contoh: 93</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Pembayaran sewa per tahun (Rp)</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="n"/>
+          <t>Frekuensi pembayaran</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n"/>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Nilai sewa setahun SEBELUM dipotong PPh. Contoh: 120.000.000</t>
+          <t>Pilih: Bulanan, Triwulanan, Semesteran, Tahunan, atau Sekaligus di awal</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
+          <t>Pembayaran sewa per periode pembayaran (Rp)</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="n"/>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Nilai SETIAP kali bayar sesuai frekuensi, SEBELUM dipotong PPh. Bila Sekaligus: total seluruh masa sewa</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
           <t>Waktu pembayaran</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Pilih: Di muka (awal tahun sewa) atau Di belakang (akhir tahun sewa)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Pilih: Di muka (awal periode bayar) atau Di belakang (akhir periode bayar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>3. BIAYA LAIN TERKAIT SEWA  (isi 0 bila tidak ada)</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="6" t="n"/>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Biaya langsung awal (Rp)</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Mis. komisi agen properti, biaya notaris kontrak sewa</t>
-        </is>
-      </c>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Pembayaran sewa di muka sebelum tanggal permulaan (Rp)</t>
+          <t>Biaya langsung awal (Rp)</t>
         </is>
       </c>
       <c r="B21" s="12" t="n"/>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Uang sewa/DP yang dibayar sebelum tanggal permulaan, di luar sewa tahunan</t>
+          <t>Mis. komisi agen properti, biaya notaris kontrak sewa</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Insentif sewa yang diterima (Rp)</t>
+          <t>Pembayaran sewa di muka sebelum tanggal permulaan (Rp)</t>
         </is>
       </c>
       <c r="B22" s="12" t="n"/>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Mis. potongan harga atau penggantian biaya dari pemilik aset</t>
+          <t>Uang sewa/DP yang dibayar sebelum tanggal permulaan, di luar sewa tahunan</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Estimasi biaya pembongkaran / restorasi (Rp)</t>
+          <t>Insentif sewa yang diterima (Rp)</t>
         </is>
       </c>
       <c r="B23" s="12" t="n"/>
       <c r="C23" s="9" t="inlineStr">
         <is>
+          <t>Mis. potongan harga atau penggantian biaya dari pemilik aset</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Estimasi biaya pembongkaran / restorasi (Rp)</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="n"/>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
           <t>Biaya mengembalikan kondisi aset di akhir sewa bila diwajibkan kontrak</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>4. INFORMASI TAMBAHAN  (boleh dikosongkan)</t>
         </is>
       </c>
-      <c r="B25" s="6" t="n"/>
-      <c r="C25" s="6" t="n"/>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Pengalihan kepemilikan / opsi beli pasti dieksekusi?</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="n"/>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>Pilih Ya bila aset akan menjadi milik Anda di akhir sewa</t>
-        </is>
-      </c>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="6" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Umur manfaat ekonomis aset (tahun)</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="n"/>
+          <t>Pengalihan kepemilikan / opsi beli pasti dieksekusi?</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="n"/>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Diperlukan bila jawaban di atas Ya. Contoh: bangunan 20, kendaraan 8</t>
+          <t>Pilih Ya bila aset akan menjadi milik Anda di akhir sewa</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
+          <t>Umur manfaat ekonomis aset (tahun)</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="n"/>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Diperlukan bila jawaban di atas Ya. Contoh: bangunan 20, kendaraan 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
           <t>Suku bunga pinjaman inkremental (% per tahun)</t>
         </is>
       </c>
-      <c r="B28" s="13" t="n"/>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="B29" s="13" t="n"/>
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t>Bunga pinjaman bank Anda untuk tenor serupa. Kosong = diisi konsultan</t>
         </is>
       </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="14" t="inlineStr">
-        <is>
-          <t>Disiapkan oleh (nama &amp; jabatan)</t>
-        </is>
-      </c>
-      <c r="B30" s="15" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
+          <t>Disiapkan oleh (nama &amp; jabatan)</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
           <t>Tanggal pengisian</t>
         </is>
       </c>
-      <c r="B31" s="16" t="n"/>
+      <c r="B32" s="16" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1"/>
-  <dataValidations count="7">
+  <dataValidations count="9">
     <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Tanah/Bangunan,Lainnya"</formula1>
     </dataValidation>
-    <dataValidation sqref="B17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Di muka (awal tahun sewa),Di belakang (akhir tahun sewa)"</formula1>
+    <dataValidation sqref="B18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Di muka (awal periode),Di belakang (akhir periode)"</formula1>
     </dataValidation>
-    <dataValidation sqref="B26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Bulanan,Triwulanan,Semesteran,Tahunan,Sekaligus di awal"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Masa sewa tidak valid" error="Isi jumlah bulan 1–600" type="whole" operator="between">
+      <formula1>1</formula1>
+      <formula2>600</formula2>
+    </dataValidation>
+    <dataValidation sqref="B27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Tidak,Ya"</formula1>
     </dataValidation>
-    <dataValidation sqref="B15 B27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Masa/umur tidak valid" error="Isi angka tahun 1–50" type="whole" operator="between">
+    <dataValidation sqref="B28" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Masa/umur tidak valid" error="Isi angka tahun 1–50" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>50</formula2>
     </dataValidation>
-    <dataValidation sqref="B16 B20 B21 B22 B23" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Isi angka rupiah (tanpa Rp/titik)" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="B17 B21 B22 B23 B24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Isi angka rupiah (tanpa Rp/titik)" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="B28" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Suku bunga tidak valid" error="Isi persen, mis. 10%" type="decimal" operator="between">
+    <dataValidation sqref="B29" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Suku bunga tidak valid" error="Isi persen, mis. 10%" type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -909,14 +929,14 @@
     <row r="6" ht="32" customHeight="1">
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>4. Pembayaran sewa per tahun adalah nilai bruto sebelum dipotong PPh Pasal 4 ayat (2) atau PPh Pasal 23.</t>
+          <t>4. Masa sewa diisi dalam bulan (mis. 93). Pembayaran diisi per kali bayar sesuai frekuensi, nilai bruto sebelum dipotong PPh Pasal 4 ayat (2) atau PPh Pasal 23.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>5. Bila sewa dibayar sekaligus untuk beberapa tahun, isi nilai per tahunnya dan pilih Waktu pembayaran 'Di muka'.</t>
+          <t>5. Bila sewa dibayar sekaligus untuk seluruh masa sewa, pilih frekuensi 'Sekaligus di awal' dan isi total nilainya.</t>
         </is>
       </c>
     </row>

</xml_diff>